<commit_message>
governance: record G-ARCH-01 and UI-00 approvals
</commit_message>
<xml_diff>
--- a/ProjectTrack_Governance_Matrix.xlsx
+++ b/ProjectTrack_Governance_Matrix.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3e29b4b586604b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Gates" sheetId="2" r:id="R8366c04c652a4eb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI UX Gates" sheetId="3" r:id="R830230e35ae84485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="4" r:id="R9e7cf395d7e946d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Matrix" sheetId="5" r:id="Rbfbc121e52654b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions" sheetId="6" r:id="R1fa4316792914876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Catalog" sheetId="7" r:id="R289b87fff2474d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkpoint Log" sheetId="8" r:id="Rc1fff3f3e6344ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R664756bacb92428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Gates" sheetId="2" r:id="R97561e1b5a2f4e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI UX Gates" sheetId="3" r:id="R7ea5e4c89c9842ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="4" r:id="R620f149cb3bd4520"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Matrix" sheetId="5" r:id="R223d3ddd5b734f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions" sheetId="6" r:id="R2612fc12908c439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Catalog" sheetId="7" r:id="R02067832d7164692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkpoint Log" sheetId="8" r:id="Ra6f7146216814886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Records" sheetId="9" r:id="Rb19058b6176d415d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,7 +45,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,6 +72,11 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -79,7 +85,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -152,14 +158,61 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="8">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -167,28 +220,7 @@
     <x:dxf>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE2F0D9"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -341,7 +373,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R49f6c3f856254d6f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc8b2590bf0aa4bb8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -475,6 +507,23 @@
     <x:tableColumn id="9" name="Evidence Path"/>
     <x:tableColumn id="10" name="Known Gaps"/>
     <x:tableColumn id="11" name="Next Permitted Step"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ApprovalRecordsTable" displayName="ApprovalRecordsTable" ref="A1:I3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Gate"/>
+    <x:tableColumn id="2" name="Decision"/>
+    <x:tableColumn id="3" name="Date"/>
+    <x:tableColumn id="4" name="Authority"/>
+    <x:tableColumn id="5" name="Reviewed Commit"/>
+    <x:tableColumn id="6" name="Conditions"/>
+    <x:tableColumn id="7" name="Record Path"/>
+    <x:tableColumn id="8" name="Exact User Response"/>
+    <x:tableColumn id="9" name="Effective Next Step"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -870,7 +919,7 @@
         <x:v>Handoff package</x:v>
       </x:c>
       <x:c r="B14" s="33" t="str">
-        <x:v>PASS</x:v>
+        <x:v>SELF-CHECK PASS / INDEPENDENT PENDING</x:v>
       </x:c>
       <x:c r="C14" s="33" t="str">
         <x:v>G-HANDOFF-00</x:v>
@@ -882,11 +931,11 @@
         <x:v>scripts/validate_handoff.py</x:v>
       </x:c>
       <x:c r="F14" s="33" t="str">
-        <x:v>Independent validation report</x:v>
-      </x:c>
-      <x:c r="G14" s="33" t="str"/>
+        <x:v>Issue formal independent verdict</x:v>
+      </x:c>
+      <x:c r="G14" s="33"/>
       <x:c r="H14" s="33" t="str">
-        <x:v>Package self-check passes</x:v>
+        <x:v>Product code remains blocked until PASS</x:v>
       </x:c>
       <x:c r="J14" t="str">
         <x:v>INT</x:v>
@@ -900,23 +949,23 @@
         <x:v>Architecture</x:v>
       </x:c>
       <x:c r="B15" s="33" t="str">
-        <x:v>NOT STARTED</x:v>
+        <x:v>APPROVED</x:v>
       </x:c>
       <x:c r="C15" s="33" t="str">
         <x:v>G-ARCH-01</x:v>
       </x:c>
       <x:c r="D15" s="33" t="str">
-        <x:v>Implementation Codex</x:v>
+        <x:v>User</x:v>
       </x:c>
       <x:c r="E15" s="33" t="str">
-        <x:v>Architecture evidence bundle</x:v>
+        <x:v>governance/approvals/G-ARCH-01_2026-09-02.md</x:v>
       </x:c>
       <x:c r="F15" s="33" t="str">
-        <x:v>Run P00/P01 only</x:v>
-      </x:c>
-      <x:c r="G15" s="33" t="str"/>
+        <x:v>Preserve approved invariants</x:v>
+      </x:c>
+      <x:c r="G15" s="33"/>
       <x:c r="H15" s="33" t="str">
-        <x:v>No product code before approval</x:v>
+        <x:v>No later architectural drift without change decision</x:v>
       </x:c>
       <x:c r="J15" t="str">
         <x:v>NFR</x:v>
@@ -930,23 +979,23 @@
         <x:v>UI information architecture</x:v>
       </x:c>
       <x:c r="B16" s="33" t="str">
-        <x:v>NOT STARTED</x:v>
+        <x:v>APPROVED</x:v>
       </x:c>
       <x:c r="C16" s="33" t="str">
         <x:v>UI-00</x:v>
       </x:c>
       <x:c r="D16" s="33" t="str">
-        <x:v>Implementation Codex + User</x:v>
+        <x:v>User</x:v>
       </x:c>
       <x:c r="E16" s="33" t="str">
-        <x:v>Low-fidelity evidence</x:v>
+        <x:v>governance/approvals/UI-00_2026-09-02.md</x:v>
       </x:c>
       <x:c r="F16" s="33" t="str">
-        <x:v>Present for user approval</x:v>
-      </x:c>
-      <x:c r="G16" s="33" t="str"/>
+        <x:v>Prepare P02 after G-HANDOFF-00 PASS</x:v>
+      </x:c>
+      <x:c r="G16" s="33"/>
       <x:c r="H16" s="33" t="str">
-        <x:v>Human approval mandatory</x:v>
+        <x:v>UI-01 remains mandatory</x:v>
       </x:c>
       <x:c r="J16" t="str">
         <x:v>GOV</x:v>
@@ -963,18 +1012,20 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="C17" s="33" t="str">
-        <x:v>G-ARCH-01 + UI-00</x:v>
+        <x:v>G-HANDOFF-00</x:v>
       </x:c>
       <x:c r="D17" s="33" t="str">
         <x:v>Implementation Codex</x:v>
       </x:c>
-      <x:c r="E17" s="33" t="str"/>
+      <x:c r="E17" s="33" t="str">
+        <x:v>CODEX_NEXT_TASK.md</x:v>
+      </x:c>
       <x:c r="F17" s="33" t="str">
-        <x:v>Wait for explicit approvals</x:v>
-      </x:c>
-      <x:c r="G17" s="33" t="str"/>
+        <x:v>Validate package, then execute P02 only</x:v>
+      </x:c>
+      <x:c r="G17" s="33"/>
       <x:c r="H17" s="33" t="str">
-        <x:v>Gate-enforced</x:v>
+        <x:v>Stop at UI-01</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -996,9 +1047,9 @@
       <x:c r="F18" s="33" t="str">
         <x:v>Connect dedicated private repository</x:v>
       </x:c>
-      <x:c r="G18" s="33" t="str"/>
+      <x:c r="G18" s="33"/>
       <x:c r="H18" s="33" t="str">
-        <x:v>Unrelated analytics repository not modified</x:v>
+        <x:v>No remote handoff confirmed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1007,7 +1058,7 @@
     <x:mergeCell ref="A12:H12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9faba3d4d234ab6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raed5913550394c45"/>
 </x:worksheet>
 </file>
 
@@ -1102,14 +1153,20 @@
         <x:v>YES</x:v>
       </x:c>
       <x:c r="F3" s="33" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>APPROVED</x:v>
       </x:c>
       <x:c r="G3" s="33" t="str">
         <x:v>Approve domain architecture, scheduling rules, data ownership and unresolved-decision register before product code.</x:v>
       </x:c>
-      <x:c r="H3" s="33" t="str"/>
-      <x:c r="I3" s="33" t="str"/>
-      <x:c r="J3" s="33" t="str"/>
+      <x:c r="H3" s="33" t="str">
+        <x:v>governance/approvals/G-ARCH-01_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="I3" s="33" t="str">
+        <x:v>G-ARCH-01_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="J3" s="33" t="str">
+        <x:v>Explicit user approval recorded; independent G-HANDOFF-00 remains pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="33" t="str">
@@ -1128,14 +1185,20 @@
         <x:v>YES</x:v>
       </x:c>
       <x:c r="F4" s="33" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>APPROVED</x:v>
       </x:c>
       <x:c r="G4" s="33" t="str">
         <x:v>Approve information architecture, command model, visual direction and All Projects concept before detailed frontend implementation.</x:v>
       </x:c>
-      <x:c r="H4" s="33" t="str"/>
-      <x:c r="I4" s="33" t="str"/>
-      <x:c r="J4" s="33" t="str"/>
+      <x:c r="H4" s="33" t="str">
+        <x:v>governance/approvals/UI-00_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="I4" s="33" t="str">
+        <x:v>UI-00_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="J4" s="33" t="str">
+        <x:v>Explicit user approval recorded; UI-01 is the next frontend gate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="33" t="str">
@@ -1510,6 +1573,11 @@
       <x:formula>OR(F2="REJECTED",F2="BLOCKED")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F3:F4">
+    <x:cfRule type="expression" dxfId="6" priority="3">
+      <x:formula>F3="APPROVED"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F2:F18">
       <x:formula1>"PENDING,IN REVIEW,APPROVED,REJECTED,CONDITIONAL,BLOCKED"</x:formula1>
@@ -1517,7 +1585,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf060f533e6e84561"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde37f930285f4719"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1587,12 +1655,20 @@
         <x:v>NO</x:v>
       </x:c>
       <x:c r="F2" s="33" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="G2" s="33" t="str"/>
-      <x:c r="H2" s="33" t="str"/>
-      <x:c r="I2" s="33" t="str"/>
-      <x:c r="J2" s="33" t="str"/>
+        <x:v>APPROVED</x:v>
+      </x:c>
+      <x:c r="G2" s="33" t="str">
+        <x:v>governance/approvals/UI-00_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="H2" s="33" t="str">
+        <x:v>APPROVE UI-00 — both gates approved; no conditions stated.</x:v>
+      </x:c>
+      <x:c r="I2" s="33" t="str">
+        <x:v>4a773b4093f9db825a0651de4f436458030bad7d</x:v>
+      </x:c>
+      <x:c r="J2" s="33" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="33" t="str">
@@ -1817,6 +1893,11 @@
     </x:cfRule>
     <x:cfRule type="expression" dxfId="3" priority="2">
       <x:formula>F2="REJECTED"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F2:F2">
+    <x:cfRule type="expression" dxfId="7" priority="3">
+      <x:formula>F2="APPROVED"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
@@ -1829,7 +1910,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R440b001bece645ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92bebe5fecf54556"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5768,7 +5849,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec2c363f74264b4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6374e0d877b4420"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5986,7 +6067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb009e829f09244b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6af76a05143541dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6641,7 +6722,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39b35a5b02744f49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R683fcfaeaa0745c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9803,7 +9884,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb030b07f404454f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re28949c17194491e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9861,17 +9942,39 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="33"/>
-      <x:c r="B2" s="33"/>
-      <x:c r="C2" s="33"/>
-      <x:c r="D2" s="33"/>
-      <x:c r="E2" s="33"/>
-      <x:c r="F2" s="33"/>
-      <x:c r="G2" s="33"/>
-      <x:c r="H2" s="33"/>
-      <x:c r="I2" s="33"/>
-      <x:c r="J2" s="33"/>
-      <x:c r="K2" s="33"/>
+      <x:c r="A2" s="33" t="str">
+        <x:v>USER-APPROVALS-2026-09-02</x:v>
+      </x:c>
+      <x:c r="B2" s="33" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="C2" s="33" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="D2" s="33" t="str">
+        <x:v>G-ARCH-01 + UI-00</x:v>
+      </x:c>
+      <x:c r="E2" s="33" t="str">
+        <x:v>4a773b4093f9db825a0651de4f436458030bad7d</x:v>
+      </x:c>
+      <x:c r="F2" s="33" t="str">
+        <x:v>No product implementation</x:v>
+      </x:c>
+      <x:c r="G2" s="33" t="str">
+        <x:v>G-HANDOFF-00 pending</x:v>
+      </x:c>
+      <x:c r="H2" s="33" t="str">
+        <x:v>APPROVED</x:v>
+      </x:c>
+      <x:c r="I2" s="33" t="str">
+        <x:v>governance/approvals/</x:v>
+      </x:c>
+      <x:c r="J2" s="33" t="str">
+        <x:v>Independent handoff validation not yet issued</x:v>
+      </x:c>
+      <x:c r="K2" s="33" t="str">
+        <x:v>Run G-HANDOFF-00; on PASS, execute P02 and stop at UI-01</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="33"/>
@@ -10524,7 +10627,119 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb57aaddd0bf4482c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R765183c70c4242ce"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="44" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="45" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="41" t="str">
+        <x:v>Gate</x:v>
+      </x:c>
+      <x:c r="B1" s="41" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="C1" s="41" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="D1" s="41" t="str">
+        <x:v>Authority</x:v>
+      </x:c>
+      <x:c r="E1" s="41" t="str">
+        <x:v>Reviewed Commit</x:v>
+      </x:c>
+      <x:c r="F1" s="41" t="str">
+        <x:v>Conditions</x:v>
+      </x:c>
+      <x:c r="G1" s="41" t="str">
+        <x:v>Record Path</x:v>
+      </x:c>
+      <x:c r="H1" s="41" t="str">
+        <x:v>Exact User Response</x:v>
+      </x:c>
+      <x:c r="I1" s="41" t="str">
+        <x:v>Effective Next Step</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="33" t="str">
+        <x:v>G-ARCH-01</x:v>
+      </x:c>
+      <x:c r="B2" s="33" t="str">
+        <x:v>APPROVED</x:v>
+      </x:c>
+      <x:c r="C2" s="33" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="D2" s="33" t="str">
+        <x:v>User</x:v>
+      </x:c>
+      <x:c r="E2" s="33" t="str">
+        <x:v>4a773b4093f9db825a0651de4f436458030bad7d</x:v>
+      </x:c>
+      <x:c r="F2" s="33" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G2" s="33" t="str">
+        <x:v>governance/approvals/G-ARCH-01_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="H2" s="33" t="str">
+        <x:v>APPROVE G-ARCH-01
+APPROVE UI-00 both are approved</x:v>
+      </x:c>
+      <x:c r="I2" s="33" t="str">
+        <x:v>Preserve approved architecture; P02 after G-HANDOFF-00 PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="33" t="str">
+        <x:v>UI-00</x:v>
+      </x:c>
+      <x:c r="B3" s="33" t="str">
+        <x:v>APPROVED</x:v>
+      </x:c>
+      <x:c r="C3" s="33" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="D3" s="33" t="str">
+        <x:v>User</x:v>
+      </x:c>
+      <x:c r="E3" s="33" t="str">
+        <x:v>4a773b4093f9db825a0651de4f436458030bad7d</x:v>
+      </x:c>
+      <x:c r="F3" s="33" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G3" s="33" t="str">
+        <x:v>governance/approvals/UI-00_2026-09-02.md</x:v>
+      </x:c>
+      <x:c r="H3" s="33" t="str">
+        <x:v>APPROVE G-ARCH-01
+APPROVE UI-00 both are approved</x:v>
+      </x:c>
+      <x:c r="I3" s="33" t="str">
+        <x:v>Build P02 shell after G-HANDOFF-00 PASS; stop at UI-01</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5e71ac129614752"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>